<commit_message>
Risk report 6/12 (signal_date 6/11): regen with split-cliff heal + authoritative NAV
The committed 6/12 risk report (040951) was doubly stale: generated 2026-06-12
04:10 BEFORE RiskManager gained heal_split_cliff (85e733c), so KLAC's root-store
weekly-cache cliff faked annual vol 360%, VaR 37.3% (false RED), and a 4.29x T_1W
balance sheet; and its NAV (1,096,917) predated the corrected strategy_performance
6/11 value. Regenerated via --as-of from combined_signals_20260612_032121
(signal_date 2026-06-11, 8-position 6/11 EOD book): NAV now 1,137,387 (authoritative),
annual vol 19.15%, VaR 1.98% (green), T_1W 2.41x. net_beta 0.9 real. KLAC heal fires
empirically at the 6/08 cache cliff. No code change — the fix was already shipped;
this only refreshes the stale artifact.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trading_signals/risk_management/risk_workbook_20260612_040951.xlsx
+++ b/trading_signals/risk_management/risk_workbook_20260612_040951.xlsx
@@ -184,22 +184,22 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -728,7 +728,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Signal date 2026-06-11  ·  Generated 2026-06-12T04:10:24  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
+          <t>Signal date 2026-06-11  ·  Generated 2026-06-14T18:46:32  ·  Scope: MRPT+MTFS pairs book (model-based, broker-reconciled)</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
     </row>
     <row r="5">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>1.09</v>
+        <v>1.051</v>
       </c>
     </row>
     <row r="6">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>0.433</v>
+        <v>0.417</v>
       </c>
     </row>
     <row r="7">
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.907</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8">
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>409308.72</v>
+        <v>22575.01</v>
       </c>
     </row>
     <row r="9">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>37.31</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="10">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>360.09</v>
+        <v>19.15</v>
       </c>
     </row>
     <row r="11">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>1.375</v>
+        <v>1.532</v>
       </c>
     </row>
     <row r="12">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>0.8532</v>
+        <v>0.8856000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8.85</v>
+        <v>8.869999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -840,7 +840,7 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>5.05 / 2.52</t>
+          <t>5.37 / 2.68</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1.09</v>
+        <v>1.051</v>
       </c>
     </row>
     <row r="16">
@@ -862,7 +862,7 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>STLD (25.84% NAV)</t>
+          <t>STLD (24.92% NAV)</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -904,7 +904,7 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>single_name_gross:STLD red</t>
+          <t>net_market_beta:combined red</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>409308.72</v>
+        <v>22575.01</v>
       </c>
     </row>
     <row r="4">
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>578755.0699999999</v>
+        <v>31920.66</v>
       </c>
     </row>
     <row r="5">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>3949893.32</v>
+        <v>217852.43</v>
       </c>
     </row>
     <row r="6">
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>360.09</v>
+        <v>19.15</v>
       </c>
     </row>
     <row r="7">
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>97304.96000000001</v>
+        <v>12071.51</v>
       </c>
     </row>
     <row r="8">
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>600838.6</v>
+        <v>20918.66</v>
       </c>
     </row>
     <row r="10">
@@ -1028,101 +1028,101 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>240081.12</v>
+        <v>6011.13</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>58.66</v>
+        <v>26.63</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>168370.15</v>
+        <v>5544.43</v>
       </c>
       <c r="C13" s="17" t="n">
-        <v>41.14</v>
+        <v>24.56</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/TRMB</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>766.9299999999999</v>
+        <v>4276.16</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>0.19</v>
+        <v>18.94</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>541.45</v>
+        <v>2440.66</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>0.13</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>507.77</v>
+        <v>1875.88</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>0.12</v>
+        <v>8.31</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="n">
-        <v>-231.4</v>
+          <t>NUE/MKTX</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>1839.39</v>
       </c>
       <c r="C17" s="17" t="n">
-        <v>-0.06</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>UNH/ULTA</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>-256.21</v>
+          <t>HST/MOS</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>446.82</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>-0.06</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
-        </is>
-      </c>
-      <c r="B19" s="18" t="n">
-        <v>-471.08</v>
+          <t>UNH/ULTA</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>140.54</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>-0.12</v>
+        <v>0.62</v>
       </c>
     </row>
   </sheetData>
@@ -1247,7 +1247,7 @@
         <v>23</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>1120096</v>
+        <v>1120098</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>0</v>
@@ -1352,7 +1352,7 @@
         <v>386</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1084241</v>
+        <v>1084242</v>
       </c>
       <c r="E13" s="17" t="n">
         <v>0</v>
@@ -1394,7 +1394,7 @@
         <v>628</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>1084241</v>
+        <v>1084242</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>0</v>
@@ -1499,7 +1499,7 @@
         <v>124</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>7011121</v>
+        <v>7011122</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>0</v>
@@ -1557,11 +1557,11 @@
           <t>SPY -5%</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
-        <v>-49745.23</v>
-      </c>
-      <c r="C4" s="23" t="n">
-        <v>-4.54</v>
+      <c r="B4" s="18" t="n">
+        <v>-51182.42</v>
+      </c>
+      <c r="C4" s="21" t="n">
+        <v>-4.5</v>
       </c>
     </row>
     <row r="5">
@@ -1570,11 +1570,11 @@
           <t>SPY -10%</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>-99490.45</v>
-      </c>
-      <c r="C5" s="21" t="n">
-        <v>-9.07</v>
+      <c r="B5" s="22" t="n">
+        <v>-102364.84</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>-9</v>
       </c>
     </row>
     <row r="6">
@@ -1583,11 +1583,11 @@
           <t>VIX +10pt</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>-49745.23</v>
-      </c>
-      <c r="C6" s="23" t="n">
-        <v>-4.54</v>
+      <c r="B6" s="18" t="n">
+        <v>-51182.42</v>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>-4.5</v>
       </c>
     </row>
     <row r="7">
@@ -1596,11 +1596,11 @@
           <t>Top sector -10%</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="22" t="n">
         <v>-45513.59</v>
       </c>
-      <c r="C7" s="21" t="n">
-        <v>-4.15</v>
+      <c r="C7" s="23" t="n">
+        <v>-4</v>
       </c>
     </row>
   </sheetData>
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="C6" s="30" t="n">
-        <v>2.27</v>
+        <v>2.07</v>
       </c>
       <c r="D6" s="30" t="n">
         <v>3</v>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="C7" s="32" t="n">
-        <v>0.9</v>
+        <v>0.82</v>
       </c>
       <c r="D7" s="32" t="n">
         <v>0.5</v>
@@ -1772,54 +1772,54 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="33" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>single_name_gross</t>
         </is>
       </c>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="32" t="inlineStr">
         <is>
           <t>STLD</t>
         </is>
       </c>
-      <c r="C8" s="34" t="n">
-        <v>25.84</v>
-      </c>
-      <c r="D8" s="34" t="n">
+      <c r="C8" s="32" t="n">
+        <v>24.92</v>
+      </c>
+      <c r="D8" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="F8" s="34" t="inlineStr">
-        <is>
-          <t>red</t>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>amber</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>single_name_gross</t>
         </is>
       </c>
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>KLAC</t>
         </is>
       </c>
-      <c r="C9" s="34" t="n">
-        <v>25.06</v>
-      </c>
-      <c r="D9" s="34" t="n">
+      <c r="C9" s="32" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="D9" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="E9" s="34" t="n">
+      <c r="E9" s="32" t="n">
         <v>25</v>
       </c>
-      <c r="F9" s="34" t="inlineStr">
-        <is>
-          <t>red</t>
+      <c r="F9" s="32" t="inlineStr">
+        <is>
+          <t>amber</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
         </is>
       </c>
       <c r="C10" s="32" t="n">
-        <v>15.65</v>
+        <v>15.09</v>
       </c>
       <c r="D10" s="32" t="n">
         <v>15</v>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="C13" s="34" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="D13" s="34" t="n">
         <v>0.3</v>
@@ -1928,28 +1928,28 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="33" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>var_95_1d</t>
         </is>
       </c>
-      <c r="B14" s="34" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>combined</t>
         </is>
       </c>
-      <c r="C14" s="34" t="n">
-        <v>37.31</v>
-      </c>
-      <c r="D14" s="34" t="n">
+      <c r="C14" s="30" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="D14" s="30" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="F14" s="34" t="inlineStr">
-        <is>
-          <t>red</t>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>green</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       <c r="F5" s="4" t="n">
         <v>611.48</v>
       </c>
-      <c r="G5" s="19" t="n">
+      <c r="G5" s="18" t="n">
         <v>-14064.04</v>
       </c>
       <c r="H5" s="7" t="inlineStr">
@@ -2248,7 +2248,7 @@
       <c r="F7" s="4" t="n">
         <v>276.91</v>
       </c>
-      <c r="G7" s="19" t="n">
+      <c r="G7" s="18" t="n">
         <v>-22706.62</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
@@ -2336,7 +2336,7 @@
       <c r="F9" s="4" t="n">
         <v>116.33</v>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>-49091.26</v>
       </c>
       <c r="H9" s="7" t="inlineStr">
@@ -2424,7 +2424,7 @@
       <c r="F11" s="4" t="n">
         <v>146.05</v>
       </c>
-      <c r="G11" s="19" t="n">
+      <c r="G11" s="18" t="n">
         <v>-52285.9</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -2512,7 +2512,7 @@
       <c r="F13" s="11" t="n">
         <v>11.27</v>
       </c>
-      <c r="G13" s="19" t="n">
+      <c r="G13" s="18" t="n">
         <v>-77120.61</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
@@ -2600,7 +2600,7 @@
       <c r="F15" s="11" t="n">
         <v>21.09</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="18" t="n">
         <v>-45723.12</v>
       </c>
       <c r="H15" s="7" t="inlineStr">
@@ -2688,7 +2688,7 @@
       <c r="F17" s="11" t="n">
         <v>50</v>
       </c>
-      <c r="G17" s="19" t="n">
+      <c r="G17" s="18" t="n">
         <v>-48600</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
@@ -2776,7 +2776,7 @@
       <c r="F19" s="4" t="n">
         <v>476.42</v>
       </c>
-      <c r="G19" s="19" t="n">
+      <c r="G19" s="18" t="n">
         <v>-50976.94</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
@@ -3091,7 +3091,7 @@
           <t>UNH/ULTA</t>
         </is>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="18" t="n">
         <v>-765.4400000000001</v>
       </c>
       <c r="D11" s="4" t="n">
@@ -3304,16 +3304,16 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>16.43</v>
+        <v>14.52</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.61</v>
+        <v>0.45</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="E6" s="23" t="n">
-        <v>-15.82</v>
+      <c r="E6" s="21" t="n">
+        <v>-14.06</v>
       </c>
     </row>
     <row r="7">
@@ -3323,16 +3323,16 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>15.19</v>
+        <v>14.93</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>17.17</v>
+        <v>29.36</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="E7" s="20" t="n">
-        <v>1.98</v>
+      <c r="E7" s="19" t="n">
+        <v>14.43</v>
       </c>
     </row>
     <row r="8">
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>27.87</v>
+        <v>25.03</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>2.27</v>
+        <v>4.02</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="E8" s="23" t="n">
-        <v>-25.6</v>
+      <c r="E8" s="21" t="n">
+        <v>-21.01</v>
       </c>
     </row>
     <row r="9">
@@ -3361,16 +3361,16 @@
         </is>
       </c>
       <c r="B9" s="17" t="n">
-        <v>40.5</v>
+        <v>45.52</v>
       </c>
       <c r="C9" s="17" t="n">
-        <v>79.94</v>
+        <v>66.17</v>
       </c>
       <c r="D9" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="E9" s="20" t="n">
-        <v>39.44</v>
+      <c r="E9" s="19" t="n">
+        <v>20.64</v>
       </c>
     </row>
     <row r="11">
@@ -3399,77 +3399,77 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>58.66</v>
+        <v>26.63</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>KLAC/TRMB</t>
+          <t>STLD/FMC</t>
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>41.14</v>
+        <v>24.56</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>NUE/INTU</t>
+          <t>KLAC/TRMB</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>0.19</v>
+        <v>18.94</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>NUE/MKTX</t>
+          <t>STLD/UHS</t>
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>0.13</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>STLD/UHS</t>
+          <t>NUE/INTU</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>0.12</v>
+        <v>8.31</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>STLD/FMC</t>
+          <t>NUE/MKTX</t>
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>-0.06</v>
+        <v>8.15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>UNH/ULTA</t>
+          <t>HST/MOS</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>-0.06</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>HST/MOS</t>
+          <t>UNH/ULTA</t>
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>-0.12</v>
+        <v>0.62</v>
       </c>
     </row>
   </sheetData>
@@ -3579,31 +3579,31 @@
           <t>COMBINED</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
-        <v>39.01</v>
+      <c r="B5" s="20" t="n">
+        <v>38.82</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>2.6</v>
+        <v>2.59</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>116</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>0.003 (t=0.04)</t>
+          <t>0.004 (t=0.04)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>-0.075 (t=-0.55)</t>
+          <t>-0.077 (t=-0.56)</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>0.072 (t=0.6)</t>
+          <t>0.074 (t=0.61)</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
@@ -3613,7 +3613,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>-0.111 (t=-0.62)</t>
+          <t>-0.109 (t=-0.61)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -3628,46 +3628,46 @@
           <t>MRPT</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
-        <v>48.72</v>
+      <c r="B6" s="19" t="n">
+        <v>45.76</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>2.02</v>
+        <v>1.8</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>116</v>
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>0.05 (t=0.36)</t>
+          <t>0.076 (t=0.51)</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>-0.109 (t=-0.5)</t>
+          <t>-0.139 (t=-0.61)</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>-0.062 (t=-0.32)</t>
+          <t>-0.053 (t=-0.26)</t>
         </is>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>0.236 (t=1.3)</t>
+          <t>0.26 (t=1.36)</t>
         </is>
       </c>
       <c r="J6" s="17" t="inlineStr">
         <is>
-          <t>-0.205 (t=-0.72)</t>
+          <t>-0.215 (t=-0.71)</t>
         </is>
       </c>
       <c r="K6" s="17" t="inlineStr">
         <is>
-          <t>-0.139 (t=-1.36)</t>
+          <t>-0.145 (t=-1.35)</t>
         </is>
       </c>
     </row>
@@ -3677,46 +3677,46 @@
           <t>MTFS</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
-        <v>27.71</v>
+      <c r="B7" s="20" t="n">
+        <v>31.8</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1.02</v>
+        <v>1.05</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.038</v>
+        <v>0.033</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>116</v>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>-0.061 (t=-0.39)</t>
+          <t>-0.096 (t=-0.54)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>-0.013 (t=-0.05)</t>
+          <t>0.029 (t=0.1)</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>0.238 (t=1.08)</t>
+          <t>0.226 (t=0.92)</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>-0.095 (t=-0.46)</t>
+          <t>-0.128 (t=-0.56)</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>0.019 (t=0.06)</t>
+          <t>0.033 (t=0.09)</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
         <is>
-          <t>-0.067 (t=-0.58)</t>
+          <t>-0.059 (t=-0.45)</t>
         </is>
       </c>
     </row>
@@ -3805,10 +3805,10 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>0.236</v>
+        <v>0.859</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>23.037</v>
+        <v>21.181</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>0</v>
@@ -3817,10 +3817,10 @@
         <v>1</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>2.25</v>
+        <v>2.416</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>2.25</v>
+        <v>2.416</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>0</v>
@@ -3833,10 +3833,10 @@
         </is>
       </c>
       <c r="B5" s="17" t="n">
-        <v>-0.313</v>
+        <v>-0.709</v>
       </c>
       <c r="C5" s="17" t="n">
-        <v>2.193</v>
+        <v>3.853</v>
       </c>
       <c r="D5" s="17" t="n">
         <v>0</v>
@@ -3845,13 +3845,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>1.57</v>
+        <v>1.648</v>
       </c>
       <c r="G5" s="17" t="n">
-        <v>1.613</v>
+        <v>1.767</v>
       </c>
       <c r="H5" s="17" t="n">
-        <v>0.043</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="6">
@@ -3861,10 +3861,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1.592</v>
+        <v>1.967</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>27.659</v>
+        <v>23.452</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0</v>
@@ -3873,10 +3873,10 @@
         <v>1</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>4.84</v>
+        <v>5.162</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>4.84</v>
+        <v>5.162</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>0</v>
@@ -3941,31 +3941,31 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>1.375</v>
+        <v>1.532</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.8532</v>
+        <v>0.8856000000000001</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>371</v>
+        <v>283</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>8.85</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>9.460000000000001</v>
+        <v>9.52</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>76.5</v>
+        <v>75.2</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>5.05</v>
+        <v>5.37</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>2.52</v>
+        <v>2.68</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>1.09</v>
+        <v>1.051</v>
       </c>
     </row>
     <row r="10">
@@ -3975,13 +3975,13 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>1.252</v>
+        <v>1.046</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>0.8300999999999999</v>
+        <v>0.7849</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>449</v>
+        <v>658</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>9.26</v>
@@ -3993,10 +3993,10 @@
         <v>77.09999999999999</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>5.9</v>
+        <v>4.49</v>
       </c>
       <c r="I10" s="17" t="n">
-        <v>2.95</v>
+        <v>2.25</v>
       </c>
       <c r="J10" s="17" t="n">
         <v>0</v>
@@ -4009,13 +4009,13 @@
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>1.074</v>
+        <v>1.315</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.8061</v>
+        <v>0.8609</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>549</v>
+        <v>349</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>15.56</v>
@@ -4024,16 +4024,16 @@
         <v>18.48</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>79.7</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>1.99</v>
+        <v>2.32</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>1</v>
+        <v>1.16</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2.269</v>
+        <v>2.073</v>
       </c>
     </row>
   </sheetData>
@@ -4108,16 +4108,16 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>254663.48</v>
+        <v>295132.72</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>165346.24</v>
+        <v>165946.58</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>117600.01</v>
+        <v>116957.77</v>
       </c>
     </row>
     <row r="6">
@@ -4152,7 +4152,7 @@
         <v>878128.87</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>3949274.76</v>
+        <v>1864541.85</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>869230.15</v>
@@ -4165,16 +4165,16 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1457486.38</v>
+        <v>1497955.62</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>1597951.19</v>
+        <v>1598551.53</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>4784167.32</v>
+        <v>2699434.41</v>
       </c>
       <c r="E8" s="13" t="n">
-        <v>1629715.98</v>
+        <v>1629073.74</v>
       </c>
     </row>
     <row r="9">
@@ -4209,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>2854249.34</v>
+        <v>768095.01</v>
       </c>
       <c r="E10" s="15" t="n">
         <v>0</v>
@@ -4228,7 +4228,7 @@
         <v>543604</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>3672771.46</v>
+        <v>1586617.13</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>630280.22</v>
@@ -4241,16 +4241,16 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>1054347.19</v>
+        <v>1054947.53</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>999435.76</v>
+        <v>998793.52</v>
       </c>
     </row>
     <row r="13">
@@ -4260,16 +4260,16 @@
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>1.09</v>
+        <v>1.051</v>
       </c>
       <c r="C13" s="7" t="n">
         <v>1.348</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>4.29</v>
+        <v>2.411</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>1.5</v>
+        <v>1.501</v>
       </c>
     </row>
     <row r="14">
@@ -4279,13 +4279,13 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>0.433</v>
+        <v>0.417</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>0.317</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>2.817</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>0.239</v>
@@ -4304,7 +4304,7 @@
         <v>284346.57</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>953559.38</v>
+        <v>536612.79</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>299902.07</v>
@@ -4317,16 +4317,16 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>857795.58</v>
+        <v>898264.8199999999</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>770000.62</v>
+        <v>770600.96</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>157836.48</v>
+        <v>576204.49</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>699533.6899999999</v>
+        <v>698891.45</v>
       </c>
     </row>
     <row r="17">
@@ -4339,7 +4339,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>0</v>
@@ -4395,7 +4395,7 @@
         <v>878128.87</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>869230.15</v>
@@ -4433,7 +4433,7 @@
         <v>878128.87</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>3949274.76</v>
+        <v>1864541.85</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>869230.15</v>
@@ -4452,7 +4452,7 @@
         <v>0</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>2837878.9</v>
+        <v>751724.5699999999</v>
       </c>
       <c r="E24" s="15" t="n">
         <v>0</v>
@@ -4471,7 +4471,7 @@
         <v>878128.87</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>869230.15</v>
@@ -4598,16 +4598,16 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>254663.48</v>
+        <v>295132.72</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>165346.24</v>
+        <v>165946.58</v>
       </c>
       <c r="D32" s="15" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E32" s="13" t="n">
-        <v>117600.01</v>
+        <v>116957.77</v>
       </c>
     </row>
     <row r="33">
@@ -4617,16 +4617,16 @@
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>1054347.19</v>
+        <v>1054947.53</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>999435.76</v>
+        <v>998793.52</v>
       </c>
     </row>
     <row r="34">
@@ -4689,16 +4689,16 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>478038.37</v>
+        <v>468816.39</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>480254.72</v>
+        <v>470884.68</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>80099.50999999999</v>
+        <v>70818.78999999999</v>
       </c>
     </row>
     <row r="40">
@@ -4746,16 +4746,16 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>744951.6899999999</v>
+        <v>735729.71</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>661799.62</v>
+        <v>652429.58</v>
       </c>
       <c r="E42" s="13" t="n">
-        <v>1081579.04</v>
+        <v>1072298.32</v>
       </c>
     </row>
     <row r="43">
@@ -4822,16 +4822,16 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C46" s="13" t="n">
-        <v>568688.47</v>
+        <v>559466.49</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>577818.58</v>
+        <v>568448.54</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>572311.02</v>
+        <v>563030.3</v>
       </c>
     </row>
     <row r="47">
@@ -4844,13 +4844,13 @@
         <v>0</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>0.463</v>
+        <v>0.471</v>
       </c>
       <c r="D47" s="7" t="n">
-        <v>0.311</v>
+        <v>0.316</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>1.732</v>
+        <v>1.761</v>
       </c>
     </row>
     <row r="48">
@@ -4863,7 +4863,7 @@
         <v>0</v>
       </c>
       <c r="C48" s="17" t="n">
-        <v>-0.157</v>
+        <v>-0.159</v>
       </c>
       <c r="D48" s="17" t="n">
         <v>0.021</v>
@@ -4898,16 +4898,16 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C50" s="13" t="n">
-        <v>516010.86</v>
+        <v>506788.88</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>541845.52</v>
+        <v>532475.48</v>
       </c>
       <c r="E50" s="13" t="n">
-        <v>374052.19</v>
+        <v>364771.47</v>
       </c>
     </row>
     <row r="51">
@@ -4926,7 +4926,7 @@
         <v>0</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -5179,16 +5179,16 @@
         </is>
       </c>
       <c r="B66" s="13" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C66" s="13" t="n">
-        <v>478038.37</v>
+        <v>468816.39</v>
       </c>
       <c r="D66" s="13" t="n">
-        <v>480254.72</v>
+        <v>470884.68</v>
       </c>
       <c r="E66" s="13" t="n">
-        <v>80099.50999999999</v>
+        <v>70818.78999999999</v>
       </c>
     </row>
     <row r="67">
@@ -5198,16 +5198,16 @@
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C67" s="4" t="n">
-        <v>568688.47</v>
+        <v>559466.49</v>
       </c>
       <c r="D67" s="4" t="n">
-        <v>577818.58</v>
+        <v>568448.54</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>572311.02</v>
+        <v>563030.3</v>
       </c>
     </row>
     <row r="68">
@@ -5279,7 +5279,7 @@
         <v>0</v>
       </c>
       <c r="E73" s="4" t="n">
-        <v>37500.5</v>
+        <v>46138.98</v>
       </c>
     </row>
     <row r="74">
@@ -5314,7 +5314,7 @@
         <v>791004.03</v>
       </c>
       <c r="D75" s="4" t="n">
-        <v>3853390.52</v>
+        <v>1768657.61</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>387204</v>
@@ -5333,10 +5333,10 @@
         <v>1165691.63</v>
       </c>
       <c r="D76" s="13" t="n">
-        <v>4602622.42</v>
+        <v>2517889.51</v>
       </c>
       <c r="E76" s="13" t="n">
-        <v>548136.9399999999</v>
+        <v>556775.42</v>
       </c>
     </row>
     <row r="77">
@@ -5365,13 +5365,13 @@
         </is>
       </c>
       <c r="B78" s="13" t="n">
-        <v>315340.38</v>
+        <v>265627.83</v>
       </c>
       <c r="C78" s="13" t="n">
-        <v>312692.13</v>
+        <v>302869.81</v>
       </c>
       <c r="D78" s="13" t="n">
-        <v>3334504.05</v>
+        <v>1238979.69</v>
       </c>
       <c r="E78" s="15" t="n">
         <v>0</v>
@@ -5384,13 +5384,13 @@
         </is>
       </c>
       <c r="B79" s="4" t="n">
-        <v>675908.87</v>
+        <v>626196.3199999999</v>
       </c>
       <c r="C79" s="4" t="n">
-        <v>680032.91</v>
+        <v>670210.59</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>4069045.13</v>
+        <v>1973520.77</v>
       </c>
       <c r="E79" s="4" t="n">
         <v>121012.2</v>
@@ -5403,16 +5403,16 @@
         </is>
       </c>
       <c r="B80" s="13" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C80" s="13" t="n">
-        <v>485658.72</v>
+        <v>495481.04</v>
       </c>
       <c r="D80" s="13" t="n">
-        <v>533577.29</v>
+        <v>544368.74</v>
       </c>
       <c r="E80" s="13" t="n">
-        <v>427124.74</v>
+        <v>435763.22</v>
       </c>
     </row>
     <row r="81">
@@ -5422,16 +5422,16 @@
         </is>
       </c>
       <c r="B81" s="7" t="n">
-        <v>2.269</v>
+        <v>2.073</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>2.385</v>
+        <v>2.338</v>
       </c>
       <c r="D81" s="7" t="n">
-        <v>8.598000000000001</v>
+        <v>4.598</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>1.19</v>
+        <v>1.166</v>
       </c>
     </row>
     <row r="82">
@@ -5441,16 +5441,16 @@
         </is>
       </c>
       <c r="B82" s="17" t="n">
-        <v>0.9</v>
+        <v>0.823</v>
       </c>
       <c r="C82" s="17" t="n">
-        <v>0.872</v>
+        <v>0.855</v>
       </c>
       <c r="D82" s="17" t="n">
-        <v>5.845</v>
+        <v>1.9</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>0.623</v>
+        <v>0.611</v>
       </c>
     </row>
     <row r="83">
@@ -5466,7 +5466,7 @@
         <v>231668.96</v>
       </c>
       <c r="D83" s="4" t="n">
-        <v>917586.3199999999</v>
+        <v>500639.74</v>
       </c>
       <c r="E83" s="4" t="n">
         <v>101643.24</v>
@@ -5479,16 +5479,16 @@
         </is>
       </c>
       <c r="B84" s="13" t="n">
-        <v>287791.72</v>
+        <v>337504.27</v>
       </c>
       <c r="C84" s="13" t="n">
-        <v>253989.76</v>
-      </c>
-      <c r="D84" s="18" t="n">
-        <v>-384009.03</v>
+        <v>263812.08</v>
+      </c>
+      <c r="D84" s="13" t="n">
+        <v>43729</v>
       </c>
       <c r="E84" s="13" t="n">
-        <v>325481.5</v>
+        <v>334119.98</v>
       </c>
     </row>
     <row r="85">
@@ -5501,7 +5501,7 @@
         <v>0</v>
       </c>
       <c r="C85" s="7" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D85" s="7" t="n">
         <v>-0</v>
@@ -5551,13 +5551,13 @@
         </is>
       </c>
       <c r="B89" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C89" s="4" t="n">
-        <v>485658.72</v>
+        <v>495481.04</v>
       </c>
       <c r="D89" s="4" t="n">
-        <v>533577.29</v>
+        <v>544368.74</v>
       </c>
       <c r="E89" s="4" t="n">
         <v>387204</v>
@@ -5595,7 +5595,7 @@
         <v>791004.03</v>
       </c>
       <c r="D91" s="4" t="n">
-        <v>3853390.52</v>
+        <v>1768657.61</v>
       </c>
       <c r="E91" s="4" t="n">
         <v>387204</v>
@@ -5608,13 +5608,13 @@
         </is>
       </c>
       <c r="B92" s="13" t="n">
-        <v>308129.01</v>
+        <v>258416.46</v>
       </c>
       <c r="C92" s="13" t="n">
-        <v>305345.31</v>
+        <v>295522.99</v>
       </c>
       <c r="D92" s="13" t="n">
-        <v>3319813.23</v>
+        <v>1224288.87</v>
       </c>
       <c r="E92" s="15" t="n">
         <v>0</v>
@@ -5627,13 +5627,13 @@
         </is>
       </c>
       <c r="B93" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C93" s="4" t="n">
-        <v>485658.72</v>
+        <v>495481.04</v>
       </c>
       <c r="D93" s="4" t="n">
-        <v>533577.29</v>
+        <v>544368.74</v>
       </c>
       <c r="E93" s="4" t="n">
         <v>387204</v>
@@ -5769,7 +5769,7 @@
         <v>0</v>
       </c>
       <c r="E100" s="13" t="n">
-        <v>37500.5</v>
+        <v>46138.98</v>
       </c>
     </row>
     <row r="101">
@@ -5779,16 +5779,16 @@
         </is>
       </c>
       <c r="B101" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C101" s="4" t="n">
-        <v>485658.72</v>
+        <v>495481.04</v>
       </c>
       <c r="D101" s="4" t="n">
-        <v>533577.29</v>
+        <v>544368.74</v>
       </c>
       <c r="E101" s="4" t="n">
-        <v>427124.74</v>
+        <v>435763.22</v>
       </c>
     </row>
     <row r="102">
@@ -5882,16 +5882,16 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>42570.7</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>-14477.97</v>
+        <v>82439.60000000001</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>24569.85</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>97482.13</v>
+        <v>138593.61</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>175419.1</v>
+        <v>215888.34</v>
       </c>
     </row>
     <row r="6">
@@ -5964,16 +5964,16 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>1315.38</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <v>-7814.73</v>
-      </c>
-      <c r="D11" s="19" t="n">
-        <v>-2307.17</v>
+        <v>1294.06</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>-7687.99</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>-2269.75</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>60671.91</v>
+        <v>51428.61</v>
       </c>
     </row>
     <row r="12">
@@ -6046,16 +6046,16 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>41255.31</v>
-      </c>
-      <c r="C17" s="19" t="n">
-        <v>-6663.26</v>
+        <v>81145.53999999999</v>
+      </c>
+      <c r="C17" s="4" t="n">
+        <v>32257.84</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>99789.28999999999</v>
+        <v>140863.36</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>114747.18</v>
+        <v>164459.73</v>
       </c>
     </row>
     <row r="18">
@@ -6065,16 +6065,16 @@
         </is>
       </c>
       <c r="B18" s="15" t="n">
-        <v>43.2</v>
+        <v>36.39</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>215.99</v>
+        <v>181.94</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>907.14</v>
+        <v>764.13</v>
       </c>
       <c r="E18" s="13" t="n">
-        <v>6609.19</v>
+        <v>5567.27</v>
       </c>
     </row>
     <row r="19">
@@ -6166,13 +6166,13 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1054347.19</v>
+        <v>1054947.53</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>999435.76</v>
+        <v>998793.52</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>921498.79</v>
@@ -6185,16 +6185,16 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>42570.7</v>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>-14477.97</v>
+        <v>82439.60000000001</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>24569.85</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>97482.13</v>
+        <v>138593.61</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>175419.1</v>
+        <v>215888.34</v>
       </c>
     </row>
     <row r="7">
@@ -6242,16 +6242,16 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
     </row>
     <row r="10">
@@ -6260,17 +6260,17 @@
           <t>Return (%)</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
-        <v>4.04</v>
-      </c>
-      <c r="C10" s="21" t="n">
-        <v>-1.3</v>
-      </c>
-      <c r="D10" s="20" t="n">
-        <v>9.75</v>
-      </c>
-      <c r="E10" s="20" t="n">
-        <v>19.04</v>
+      <c r="B10" s="19" t="n">
+        <v>7.81</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>2.21</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>23.43</v>
       </c>
     </row>
     <row r="11">
@@ -6279,17 +6279,17 @@
           <t>Max drawdown (%)</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="23" t="n">
-        <v>-9.359999999999999</v>
-      </c>
-      <c r="D11" s="23" t="n">
-        <v>-9.359999999999999</v>
-      </c>
-      <c r="E11" s="23" t="n">
-        <v>-9.460000000000001</v>
+      <c r="B11" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="21" t="n">
+        <v>-9.52</v>
+      </c>
+      <c r="D11" s="21" t="n">
+        <v>-9.52</v>
+      </c>
+      <c r="E11" s="21" t="n">
+        <v>-9.52</v>
       </c>
     </row>
     <row r="13">
@@ -6333,13 +6333,13 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>568688.47</v>
+        <v>559466.49</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>577818.58</v>
+        <v>568448.54</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>572311.02</v>
+        <v>563030.3</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>509331.94</v>
@@ -6352,16 +6352,16 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1315.38</v>
-      </c>
-      <c r="C16" s="18" t="n">
-        <v>-7814.73</v>
-      </c>
-      <c r="D16" s="18" t="n">
-        <v>-2307.17</v>
+        <v>1294.06</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>-7687.99</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>-2269.75</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>60671.91</v>
+        <v>51428.61</v>
       </c>
     </row>
     <row r="17">
@@ -6409,16 +6409,16 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
     </row>
     <row r="20">
@@ -6427,17 +6427,17 @@
           <t>Return (%)</t>
         </is>
       </c>
-      <c r="B20" s="20" t="n">
+      <c r="B20" s="19" t="n">
         <v>0.23</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="23" t="n">
         <v>-1.35</v>
       </c>
-      <c r="D20" s="21" t="n">
+      <c r="D20" s="23" t="n">
         <v>-0.4</v>
       </c>
-      <c r="E20" s="20" t="n">
-        <v>11.91</v>
+      <c r="E20" s="19" t="n">
+        <v>10.1</v>
       </c>
     </row>
     <row r="21">
@@ -6446,16 +6446,16 @@
           <t>Max drawdown (%)</t>
         </is>
       </c>
-      <c r="B21" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="23" t="n">
+      <c r="B21" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="21" t="n">
         <v>-1.58</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="21" t="n">
         <v>-3.55</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="21" t="n">
         <v>-9.57</v>
       </c>
     </row>
@@ -6500,13 +6500,13 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>485658.72</v>
+        <v>495481.04</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>533577.29</v>
+        <v>544368.74</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>427124.74</v>
+        <v>435763.22</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>412166.85</v>
@@ -6519,16 +6519,16 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>41255.31</v>
-      </c>
-      <c r="C26" s="18" t="n">
-        <v>-6663.26</v>
+        <v>81145.53999999999</v>
+      </c>
+      <c r="C26" s="13" t="n">
+        <v>32257.84</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>99789.28999999999</v>
+        <v>140863.36</v>
       </c>
       <c r="E26" s="13" t="n">
-        <v>114747.18</v>
+        <v>164459.73</v>
       </c>
     </row>
     <row r="27">
@@ -6576,16 +6576,16 @@
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
     </row>
     <row r="30">
@@ -6594,17 +6594,17 @@
           <t>Return (%)</t>
         </is>
       </c>
-      <c r="B30" s="20" t="n">
-        <v>8.49</v>
-      </c>
-      <c r="C30" s="21" t="n">
-        <v>-1.25</v>
-      </c>
-      <c r="D30" s="20" t="n">
-        <v>23.36</v>
-      </c>
-      <c r="E30" s="20" t="n">
-        <v>27.84</v>
+      <c r="B30" s="19" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="C30" s="19" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="D30" s="19" t="n">
+        <v>32.33</v>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>39.9</v>
       </c>
     </row>
     <row r="31">
@@ -6613,16 +6613,16 @@
           <t>Max drawdown (%)</t>
         </is>
       </c>
-      <c r="B31" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C31" s="23" t="n">
+      <c r="B31" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="21" t="n">
         <v>-18.48</v>
       </c>
-      <c r="D31" s="23" t="n">
+      <c r="D31" s="21" t="n">
         <v>-18.48</v>
       </c>
-      <c r="E31" s="23" t="n">
+      <c r="E31" s="21" t="n">
         <v>-18.48</v>
       </c>
     </row>
@@ -6672,8 +6672,8 @@
           <t>Operating cash flow</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
-        <v>-14477.97</v>
+      <c r="B4" s="4" t="n">
+        <v>24569.85</v>
       </c>
     </row>
     <row r="5">
@@ -6683,7 +6683,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>2656278.09</v>
+        <v>571545.1800000001</v>
       </c>
     </row>
     <row r="6">
@@ -6692,8 +6692,8 @@
           <t>Financing cash flow</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n">
-        <v>-2854249.34</v>
+      <c r="B6" s="18" t="n">
+        <v>-768095.01</v>
       </c>
     </row>
     <row r="7">
@@ -6702,8 +6702,8 @@
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n">
-        <v>-212449.22</v>
+      <c r="B7" s="18" t="n">
+        <v>-171979.98</v>
       </c>
     </row>
     <row r="8">
@@ -6723,7 +6723,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>254663.48</v>
+        <v>295132.72</v>
       </c>
     </row>
     <row r="11">
@@ -7700,7 +7700,7 @@
         </is>
       </c>
       <c r="B96" s="4" t="n">
-        <v>1011251.3</v>
+        <v>1011103.74</v>
       </c>
     </row>
     <row r="97">
@@ -7710,7 +7710,7 @@
         </is>
       </c>
       <c r="B97" s="13" t="n">
-        <v>1025508.62</v>
+        <v>1025051.32</v>
       </c>
     </row>
     <row r="98">
@@ -7720,7 +7720,7 @@
         </is>
       </c>
       <c r="B98" s="4" t="n">
-        <v>1027012.9</v>
+        <v>1026690.72</v>
       </c>
     </row>
     <row r="99">
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="B99" s="13" t="n">
-        <v>1015229.96</v>
+        <v>1015359.98</v>
       </c>
     </row>
     <row r="100">
@@ -7740,7 +7740,7 @@
         </is>
       </c>
       <c r="B100" s="4" t="n">
-        <v>1002957.48</v>
+        <v>1003162.43</v>
       </c>
     </row>
     <row r="101">
@@ -7750,7 +7750,7 @@
         </is>
       </c>
       <c r="B101" s="13" t="n">
-        <v>1013008.53</v>
+        <v>1013277.95</v>
       </c>
     </row>
     <row r="102">
@@ -7760,7 +7760,7 @@
         </is>
       </c>
       <c r="B102" s="4" t="n">
-        <v>1026566.99</v>
+        <v>1027021.03</v>
       </c>
     </row>
     <row r="103">
@@ -7770,7 +7770,7 @@
         </is>
       </c>
       <c r="B103" s="13" t="n">
-        <v>1053183.37</v>
+        <v>1054148.08</v>
       </c>
     </row>
     <row r="104">
@@ -7780,7 +7780,7 @@
         </is>
       </c>
       <c r="B104" s="4" t="n">
-        <v>1050518.31</v>
+        <v>1051498.27</v>
       </c>
     </row>
     <row r="105">
@@ -7790,7 +7790,7 @@
         </is>
       </c>
       <c r="B105" s="13" t="n">
-        <v>1049333.4</v>
+        <v>1050078.94</v>
       </c>
     </row>
     <row r="106">
@@ -7800,7 +7800,7 @@
         </is>
       </c>
       <c r="B106" s="4" t="n">
-        <v>1049004.36</v>
+        <v>1049591.92</v>
       </c>
     </row>
     <row r="107">
@@ -7810,7 +7810,7 @@
         </is>
       </c>
       <c r="B107" s="13" t="n">
-        <v>1042828.15</v>
+        <v>1043241.05</v>
       </c>
     </row>
     <row r="108">
@@ -7820,7 +7820,7 @@
         </is>
       </c>
       <c r="B108" s="4" t="n">
-        <v>1048588.91</v>
+        <v>1049025.46</v>
       </c>
     </row>
     <row r="109">
@@ -7830,7 +7830,7 @@
         </is>
       </c>
       <c r="B109" s="13" t="n">
-        <v>1042675.19</v>
+        <v>1043117.12</v>
       </c>
     </row>
     <row r="110">
@@ -7840,7 +7840,7 @@
         </is>
       </c>
       <c r="B110" s="4" t="n">
-        <v>1044121.69</v>
+        <v>1044635.34</v>
       </c>
     </row>
     <row r="111">
@@ -7850,7 +7850,7 @@
         </is>
       </c>
       <c r="B111" s="13" t="n">
-        <v>1070244.76</v>
+        <v>1070736.97</v>
       </c>
     </row>
     <row r="112">
@@ -7860,7 +7860,7 @@
         </is>
       </c>
       <c r="B112" s="4" t="n">
-        <v>1061425.68</v>
+        <v>1061826.91</v>
       </c>
     </row>
     <row r="113">
@@ -7870,7 +7870,7 @@
         </is>
       </c>
       <c r="B113" s="13" t="n">
-        <v>1074852.68</v>
+        <v>1074933.41</v>
       </c>
     </row>
     <row r="114">
@@ -7880,7 +7880,7 @@
         </is>
       </c>
       <c r="B114" s="4" t="n">
-        <v>1080530.48</v>
+        <v>1080449.67</v>
       </c>
     </row>
     <row r="115">
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="B115" s="13" t="n">
-        <v>1086984.11</v>
+        <v>1086715.78</v>
       </c>
     </row>
     <row r="116">
@@ -7900,7 +7900,7 @@
         </is>
       </c>
       <c r="B116" s="4" t="n">
-        <v>1071748.22</v>
+        <v>1071892.67</v>
       </c>
     </row>
     <row r="117">
@@ -7910,7 +7910,7 @@
         </is>
       </c>
       <c r="B117" s="13" t="n">
-        <v>1065532.89</v>
+        <v>1065502.29</v>
       </c>
     </row>
     <row r="118">
@@ -7920,7 +7920,7 @@
         </is>
       </c>
       <c r="B118" s="4" t="n">
-        <v>1080655.62</v>
+        <v>1080379.78</v>
       </c>
     </row>
     <row r="119">
@@ -7930,7 +7930,7 @@
         </is>
       </c>
       <c r="B119" s="13" t="n">
-        <v>1075694.44</v>
+        <v>1075233.42</v>
       </c>
     </row>
     <row r="120">
@@ -7940,7 +7940,7 @@
         </is>
       </c>
       <c r="B120" s="4" t="n">
-        <v>1071136.6</v>
+        <v>1070583.4</v>
       </c>
     </row>
     <row r="121">
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="B121" s="13" t="n">
-        <v>1073844.08</v>
+        <v>1073148.35</v>
       </c>
     </row>
     <row r="122">
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="B122" s="4" t="n">
-        <v>1074388.79</v>
+        <v>1073704.08</v>
       </c>
     </row>
     <row r="123">
@@ -7970,7 +7970,7 @@
         </is>
       </c>
       <c r="B123" s="13" t="n">
-        <v>1084719.96</v>
+        <v>1083942.34</v>
       </c>
     </row>
     <row r="124">
@@ -7980,7 +7980,7 @@
         </is>
       </c>
       <c r="B124" s="4" t="n">
-        <v>1085696.79</v>
+        <v>1084938.93</v>
       </c>
     </row>
     <row r="125">
@@ -7990,7 +7990,7 @@
         </is>
       </c>
       <c r="B125" s="13" t="n">
-        <v>1092785.32</v>
+        <v>1092024.86</v>
       </c>
     </row>
     <row r="126">
@@ -8000,7 +8000,7 @@
         </is>
       </c>
       <c r="B126" s="4" t="n">
-        <v>1092961.6</v>
+        <v>1092149.17</v>
       </c>
     </row>
     <row r="127">
@@ -8010,7 +8010,7 @@
         </is>
       </c>
       <c r="B127" s="13" t="n">
-        <v>1053693.85</v>
+        <v>1052087.23</v>
       </c>
     </row>
     <row r="128">
@@ -8020,7 +8020,7 @@
         </is>
       </c>
       <c r="B128" s="4" t="n">
-        <v>1050036.71</v>
+        <v>1048464.49</v>
       </c>
     </row>
     <row r="129">
@@ -8030,7 +8030,7 @@
         </is>
       </c>
       <c r="B129" s="13" t="n">
-        <v>1044428.24</v>
+        <v>1042951.71</v>
       </c>
     </row>
     <row r="130">
@@ -8040,7 +8040,7 @@
         </is>
       </c>
       <c r="B130" s="4" t="n">
-        <v>1032935.01</v>
+        <v>1031548.19</v>
       </c>
     </row>
     <row r="131">
@@ -8050,7 +8050,7 @@
         </is>
       </c>
       <c r="B131" s="13" t="n">
-        <v>1039988.89</v>
+        <v>1038690.65</v>
       </c>
     </row>
     <row r="132">
@@ -8060,7 +8060,7 @@
         </is>
       </c>
       <c r="B132" s="4" t="n">
-        <v>1037824.8</v>
+        <v>1036595.47</v>
       </c>
     </row>
     <row r="133">
@@ -8070,7 +8070,7 @@
         </is>
       </c>
       <c r="B133" s="13" t="n">
-        <v>1019545.9</v>
+        <v>1018492.18</v>
       </c>
     </row>
     <row r="134">
@@ -8080,7 +8080,7 @@
         </is>
       </c>
       <c r="B134" s="4" t="n">
-        <v>1014353.52</v>
+        <v>1013499.62</v>
       </c>
     </row>
     <row r="135">
@@ -8090,7 +8090,7 @@
         </is>
       </c>
       <c r="B135" s="13" t="n">
-        <v>999435.76</v>
+        <v>998793.52</v>
       </c>
     </row>
     <row r="136">
@@ -8100,7 +8100,7 @@
         </is>
       </c>
       <c r="B136" s="4" t="n">
-        <v>1011607</v>
+        <v>1010719.54</v>
       </c>
     </row>
     <row r="137">
@@ -8110,7 +8110,7 @@
         </is>
       </c>
       <c r="B137" s="13" t="n">
-        <v>1014754.63</v>
+        <v>1013792.37</v>
       </c>
     </row>
     <row r="138">
@@ -8120,7 +8120,7 @@
         </is>
       </c>
       <c r="B138" s="4" t="n">
-        <v>1012093.49</v>
+        <v>1011137.79</v>
       </c>
     </row>
     <row r="139">
@@ -8130,7 +8130,7 @@
         </is>
       </c>
       <c r="B139" s="13" t="n">
-        <v>998605.65</v>
+        <v>997749.49</v>
       </c>
     </row>
     <row r="140">
@@ -8140,7 +8140,7 @@
         </is>
       </c>
       <c r="B140" s="4" t="n">
-        <v>1014471.67</v>
+        <v>1013932.08</v>
       </c>
     </row>
     <row r="141">
@@ -8150,7 +8150,7 @@
         </is>
       </c>
       <c r="B141" s="13" t="n">
-        <v>1023635.34</v>
+        <v>1023020.78</v>
       </c>
     </row>
     <row r="142">
@@ -8160,7 +8160,7 @@
         </is>
       </c>
       <c r="B142" s="4" t="n">
-        <v>1023795.45</v>
+        <v>1023350.89</v>
       </c>
     </row>
     <row r="143">
@@ -8170,7 +8170,7 @@
         </is>
       </c>
       <c r="B143" s="13" t="n">
-        <v>997080.27</v>
+        <v>996212.58</v>
       </c>
     </row>
     <row r="144">
@@ -8180,7 +8180,7 @@
         </is>
       </c>
       <c r="B144" s="4" t="n">
-        <v>1016630.21</v>
+        <v>1016375.33</v>
       </c>
     </row>
     <row r="145">
@@ -8190,7 +8190,7 @@
         </is>
       </c>
       <c r="B145" s="13" t="n">
-        <v>997982.37</v>
+        <v>997437.28</v>
       </c>
     </row>
     <row r="146">
@@ -8200,7 +8200,7 @@
         </is>
       </c>
       <c r="B146" s="4" t="n">
-        <v>991680.36</v>
+        <v>990840.4</v>
       </c>
     </row>
     <row r="147">
@@ -8210,7 +8210,7 @@
         </is>
       </c>
       <c r="B147" s="13" t="n">
-        <v>989575.49</v>
+        <v>988548.85</v>
       </c>
     </row>
     <row r="148">
@@ -8220,7 +8220,7 @@
         </is>
       </c>
       <c r="B148" s="4" t="n">
-        <v>1005081.05</v>
+        <v>1004260.13</v>
       </c>
     </row>
     <row r="149">
@@ -8230,7 +8230,7 @@
         </is>
       </c>
       <c r="B149" s="13" t="n">
-        <v>1099409.95</v>
+        <v>1100523.26</v>
       </c>
     </row>
     <row r="150">
@@ -8240,7 +8240,7 @@
         </is>
       </c>
       <c r="B150" s="4" t="n">
-        <v>1108135.74</v>
+        <v>1109402.67</v>
       </c>
     </row>
     <row r="151">
@@ -8250,7 +8250,7 @@
         </is>
       </c>
       <c r="B151" s="13" t="n">
-        <v>1111395.86</v>
+        <v>1112817.28</v>
       </c>
     </row>
     <row r="152">
@@ -8260,7 +8260,7 @@
         </is>
       </c>
       <c r="B152" s="4" t="n">
-        <v>1007363.38</v>
+        <v>1006878.56</v>
       </c>
     </row>
     <row r="153">
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="B153" s="13" t="n">
-        <v>1063573.9</v>
+        <v>1064254.6</v>
       </c>
     </row>
     <row r="154">
@@ -8280,7 +8280,7 @@
         </is>
       </c>
       <c r="B154" s="4" t="n">
-        <v>1055499.9</v>
+        <v>1056068.38</v>
       </c>
     </row>
     <row r="155">
@@ -8290,7 +8290,7 @@
         </is>
       </c>
       <c r="B155" s="13" t="n">
-        <v>1054347.19</v>
+        <v>1054947.53</v>
       </c>
     </row>
     <row r="156">
@@ -8300,7 +8300,7 @@
         </is>
       </c>
       <c r="B156" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
     </row>
   </sheetData>
@@ -8405,7 +8405,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1096917.89</v>
+        <v>1137387.13</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>835043.04</v>
@@ -8420,16 +8420,16 @@
         <v>474474.55</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>1.09</v>
+        <v>1.051</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>0.433</v>
+        <v>0.417</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>109</v>
+        <v>105.12</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>54.5</v>
+        <v>52.56</v>
       </c>
       <c r="K4" s="24" t="n">
         <v>8</v>
@@ -8442,7 +8442,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>570003.85</v>
+        <v>560760.55</v>
       </c>
       <c r="C5" s="15" t="n">
         <v>0</v>
@@ -8479,7 +8479,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>526914.03</v>
+        <v>576626.58</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>835043.04</v>
@@ -8494,16 +8494,16 @@
         <v>474474.55</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>2.269</v>
+        <v>2.073</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.9</v>
+        <v>0.823</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>226.91</v>
+        <v>207.35</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>113.45</v>
+        <v>103.67</v>
       </c>
       <c r="K6" s="24" t="n">
         <v>8</v>
@@ -8592,10 +8592,10 @@
       <c r="C6" s="4" t="n">
         <v>283463.7</v>
       </c>
-      <c r="D6" s="22" t="n">
-        <v>25.84</v>
-      </c>
-      <c r="E6" s="22" t="n">
+      <c r="D6" s="20" t="n">
+        <v>24.92</v>
+      </c>
+      <c r="E6" s="20" t="n">
         <v>23.71</v>
       </c>
       <c r="F6" s="24" t="n">
@@ -8614,10 +8614,10 @@
       <c r="C7" s="13" t="n">
         <v>274926.96</v>
       </c>
-      <c r="D7" s="20" t="n">
-        <v>25.06</v>
-      </c>
-      <c r="E7" s="20" t="n">
+      <c r="D7" s="19" t="n">
+        <v>24.17</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>22.99</v>
       </c>
       <c r="F7" s="26" t="n">
@@ -8636,10 +8636,10 @@
       <c r="C8" s="4" t="n">
         <v>171672.2</v>
       </c>
-      <c r="D8" s="22" t="n">
-        <v>15.65</v>
-      </c>
-      <c r="E8" s="22" t="n">
+      <c r="D8" s="20" t="n">
+        <v>15.09</v>
+      </c>
+      <c r="E8" s="20" t="n">
         <v>14.36</v>
       </c>
       <c r="F8" s="24" t="n">
@@ -8655,13 +8655,13 @@
       <c r="B9" s="13" t="n">
         <v>77120.61</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="22" t="n">
         <v>-77120.61</v>
       </c>
-      <c r="D9" s="20" t="n">
-        <v>7.03</v>
-      </c>
-      <c r="E9" s="20" t="n">
+      <c r="D9" s="19" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>6.45</v>
       </c>
       <c r="F9" s="26" t="n">
@@ -8680,10 +8680,10 @@
       <c r="C10" s="4" t="n">
         <v>54691.98</v>
       </c>
-      <c r="D10" s="22" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="E10" s="22" t="n">
+      <c r="D10" s="20" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="E10" s="20" t="n">
         <v>4.57</v>
       </c>
       <c r="F10" s="24" t="n">
@@ -8699,13 +8699,13 @@
       <c r="B11" s="13" t="n">
         <v>52285.9</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="22" t="n">
         <v>-52285.9</v>
       </c>
-      <c r="D11" s="20" t="n">
-        <v>4.77</v>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="D11" s="19" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>4.37</v>
       </c>
       <c r="F11" s="26" t="n">
@@ -8721,13 +8721,13 @@
       <c r="B12" s="4" t="n">
         <v>50976.94</v>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="18" t="n">
         <v>-50976.94</v>
       </c>
-      <c r="D12" s="22" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="E12" s="22" t="n">
+      <c r="D12" s="20" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>4.26</v>
       </c>
       <c r="F12" s="24" t="n">
@@ -8746,10 +8746,10 @@
       <c r="C13" s="13" t="n">
         <v>50288.2</v>
       </c>
-      <c r="D13" s="20" t="n">
-        <v>4.58</v>
-      </c>
-      <c r="E13" s="20" t="n">
+      <c r="D13" s="19" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="E13" s="19" t="n">
         <v>4.21</v>
       </c>
       <c r="F13" s="26" t="n">
@@ -8765,13 +8765,13 @@
       <c r="B14" s="4" t="n">
         <v>49091.26</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="18" t="n">
         <v>-49091.26</v>
       </c>
-      <c r="D14" s="22" t="n">
-        <v>4.48</v>
-      </c>
-      <c r="E14" s="22" t="n">
+      <c r="D14" s="20" t="n">
+        <v>4.32</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <v>4.11</v>
       </c>
       <c r="F14" s="24" t="n">
@@ -8787,13 +8787,13 @@
       <c r="B15" s="13" t="n">
         <v>48600</v>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="22" t="n">
         <v>-48600</v>
       </c>
-      <c r="D15" s="20" t="n">
-        <v>4.43</v>
-      </c>
-      <c r="E15" s="20" t="n">
+      <c r="D15" s="19" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="E15" s="19" t="n">
         <v>4.06</v>
       </c>
       <c r="F15" s="26" t="n">
@@ -8884,7 +8884,7 @@
       <c r="C22" s="4" t="n">
         <v>173820.67</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="18" t="n">
         <v>-173820.67</v>
       </c>
       <c r="E22" s="7" t="n">
@@ -8922,7 +8922,7 @@
       <c r="C24" s="4" t="n">
         <v>48600</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="18" t="n">
         <v>-48600</v>
       </c>
       <c r="E24" s="7" t="n">
@@ -8941,7 +8941,7 @@
       <c r="C25" s="13" t="n">
         <v>66349.94</v>
       </c>
-      <c r="D25" s="18" t="n">
+      <c r="D25" s="22" t="n">
         <v>-16061.74</v>
       </c>
       <c r="E25" s="17" t="n">
@@ -8983,7 +8983,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.907</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4">
@@ -8993,7 +8993,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1.375</v>
+        <v>1.351</v>
       </c>
     </row>
     <row r="5">
@@ -9003,7 +9003,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>43.26</v>
+        <v>41.72</v>
       </c>
     </row>
     <row r="6">
@@ -9043,7 +9043,7 @@
           <t>materials</t>
         </is>
       </c>
-      <c r="B10" s="22" t="n">
+      <c r="B10" s="20" t="n">
         <v>38.07</v>
       </c>
     </row>
@@ -9053,7 +9053,7 @@
           <t>tech</t>
         </is>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="19" t="n">
         <v>16.99</v>
       </c>
     </row>
@@ -9063,7 +9063,7 @@
           <t>food</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="21" t="n">
         <v>-14.54</v>
       </c>
     </row>
@@ -9073,7 +9073,7 @@
           <t>realestate</t>
         </is>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="19" t="n">
         <v>4.57</v>
       </c>
     </row>
@@ -9083,7 +9083,7 @@
           <t>industrial</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="21" t="n">
         <v>-4.06</v>
       </c>
     </row>
@@ -9093,7 +9093,7 @@
           <t>health</t>
         </is>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="23" t="n">
         <v>-1.34</v>
       </c>
     </row>

</xml_diff>